<commit_message>
Added new RDF data schemes and visual schemes for economy-table126-129, fixed XLSX spreadsheets for economy-table126-128
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table126.xlsx
+++ b/sources/table_normalization/xlsx/economy-table126.xlsx
@@ -112,11 +112,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="5">
-    <numFmt numFmtId="168" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
-    <numFmt numFmtId="169" formatCode="0.0"/>
-    <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="171" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="172" formatCode="_-* #,##0.00\ [$₽-419]_-;\-* #,##0.00\ [$₽-419]_-;_-* &quot;-&quot;??\ [$₽-419]_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="168" formatCode="_-* #,##0.00\ [$₽-419]_-;\-* #,##0.00\ [$₽-419]_-;_-* &quot;-&quot;??\ [$₽-419]_-;_-@_-"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -239,7 +239,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -255,6 +255,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -605,7 +611,7 @@
     <xf numFmtId="1" fontId="8" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="8" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -618,71 +624,41 @@
     <xf numFmtId="1" fontId="8" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="8" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="170" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="8" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="8" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="171" fontId="8" fillId="0" borderId="16" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="16" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="170" fontId="8" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="8" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="171" fontId="8" fillId="0" borderId="17" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="17" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="6" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="8" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="10" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="2" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="15" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="5" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -698,22 +674,13 @@
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="170" fontId="1" fillId="3" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="1" fillId="3" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="171" fontId="6" fillId="3" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="6" fillId="3" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="170" fontId="3" fillId="2" borderId="13" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="2" fillId="2" borderId="13" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="2" fillId="2" borderId="18" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -734,8 +701,47 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="3" fillId="0" borderId="13" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="13" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="8" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="10" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="4" borderId="13" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="13" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="18" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="3" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1228,27 +1234,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="31">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="63" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="2"/>
-      <c r="D1" s="44" t="s">
+      <c r="D1" s="36" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="14"/>
       <c r="F1" s="15"/>
       <c r="G1" s="16"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
+      <c r="H1" s="57"/>
+      <c r="I1" s="57"/>
       <c r="J1" s="28"/>
-      <c r="K1" s="45" t="s">
+      <c r="K1" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="45"/>
+      <c r="L1" s="61"/>
     </row>
     <row r="2" spans="1:12" ht="17">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="64" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="1"/>
@@ -1260,51 +1266,51 @@
       <c r="H2" s="4"/>
       <c r="I2" s="29"/>
       <c r="J2" s="29"/>
-      <c r="K2" s="46" t="s">
+      <c r="K2" s="62" t="s">
         <v>4</v>
       </c>
-      <c r="L2" s="46"/>
+      <c r="L2" s="62"/>
     </row>
     <row r="3" spans="1:12" ht="39">
-      <c r="A3" s="47" t="s">
+      <c r="A3" s="37" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="48" t="s">
+      <c r="B3" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="49" t="s">
+      <c r="C3" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="49" t="s">
+      <c r="D3" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="50" t="s">
+      <c r="E3" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="51" t="s">
+      <c r="F3" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="48" t="s">
+      <c r="G3" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="49" t="s">
+      <c r="H3" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="I3" s="52" t="s">
+      <c r="I3" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="J3" s="52" t="s">
+      <c r="J3" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="K3" s="53" t="s">
+      <c r="K3" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="L3" s="53" t="s">
+      <c r="L3" s="43" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="15.5">
-      <c r="A4" s="37">
+      <c r="A4" s="54">
         <v>42036</v>
       </c>
       <c r="B4" s="5">
@@ -1342,7 +1348,7 @@
       </c>
     </row>
     <row r="5" spans="1:12" ht="15.5">
-      <c r="A5" s="37"/>
+      <c r="A5" s="54"/>
       <c r="B5" s="8">
         <v>49622</v>
       </c>
@@ -1378,7 +1384,7 @@
       </c>
     </row>
     <row r="6" spans="1:12" ht="15.5">
-      <c r="A6" s="37"/>
+      <c r="A6" s="54"/>
       <c r="B6" s="8">
         <v>49623</v>
       </c>
@@ -1414,7 +1420,7 @@
       </c>
     </row>
     <row r="7" spans="1:12" ht="15.5">
-      <c r="A7" s="37"/>
+      <c r="A7" s="54"/>
       <c r="B7" s="8">
         <v>49624</v>
       </c>
@@ -1450,7 +1456,7 @@
       </c>
     </row>
     <row r="8" spans="1:12" ht="15.5">
-      <c r="A8" s="37"/>
+      <c r="A8" s="54"/>
       <c r="B8" s="8">
         <v>49625</v>
       </c>
@@ -1486,7 +1492,7 @@
       </c>
     </row>
     <row r="9" spans="1:12" ht="15.5">
-      <c r="A9" s="37"/>
+      <c r="A9" s="54"/>
       <c r="B9" s="8">
         <v>49926</v>
       </c>
@@ -1522,7 +1528,7 @@
       </c>
     </row>
     <row r="10" spans="1:12" ht="15.5">
-      <c r="A10" s="38"/>
+      <c r="A10" s="53"/>
       <c r="B10" s="8">
         <v>49927</v>
       </c>
@@ -1558,7 +1564,7 @@
       </c>
     </row>
     <row r="11" spans="1:12" ht="15.5">
-      <c r="A11" s="39">
+      <c r="A11" s="52">
         <v>42037</v>
       </c>
       <c r="B11" s="8">
@@ -1596,7 +1602,7 @@
       </c>
     </row>
     <row r="12" spans="1:12" ht="15.5">
-      <c r="A12" s="37"/>
+      <c r="A12" s="54"/>
       <c r="B12" s="8">
         <v>49929</v>
       </c>
@@ -1632,7 +1638,7 @@
       </c>
     </row>
     <row r="13" spans="1:12" ht="15.5">
-      <c r="A13" s="38"/>
+      <c r="A13" s="53"/>
       <c r="B13" s="8">
         <v>49930</v>
       </c>
@@ -1668,7 +1674,7 @@
       </c>
     </row>
     <row r="14" spans="1:12" ht="15.5">
-      <c r="A14" s="39">
+      <c r="A14" s="52">
         <v>42040</v>
       </c>
       <c r="B14" s="12">
@@ -1706,7 +1712,7 @@
       </c>
     </row>
     <row r="15" spans="1:12" ht="15.5">
-      <c r="A15" s="38"/>
+      <c r="A15" s="53"/>
       <c r="B15" s="12">
         <v>762479</v>
       </c>
@@ -1742,7 +1748,7 @@
       </c>
     </row>
     <row r="16" spans="1:12" ht="15.5">
-      <c r="A16" s="39">
+      <c r="A16" s="52">
         <v>42041</v>
       </c>
       <c r="B16" s="12">
@@ -1780,7 +1786,7 @@
       </c>
     </row>
     <row r="17" spans="1:12" ht="15.5">
-      <c r="A17" s="37"/>
+      <c r="A17" s="54"/>
       <c r="B17" s="12">
         <v>762481</v>
       </c>
@@ -1816,7 +1822,7 @@
       </c>
     </row>
     <row r="18" spans="1:12" ht="15.5">
-      <c r="A18" s="38"/>
+      <c r="A18" s="53"/>
       <c r="B18" s="12">
         <v>762482</v>
       </c>
@@ -1852,7 +1858,7 @@
       </c>
     </row>
     <row r="19" spans="1:12" ht="15.5">
-      <c r="A19" s="40">
+      <c r="A19" s="55">
         <v>42042</v>
       </c>
       <c r="B19" s="13">
@@ -1890,7 +1896,7 @@
       </c>
     </row>
     <row r="20" spans="1:12" ht="15.5">
-      <c r="A20" s="41"/>
+      <c r="A20" s="56"/>
       <c r="B20" s="13">
         <v>49932</v>
       </c>
@@ -1926,7 +1932,7 @@
       </c>
     </row>
     <row r="21" spans="1:12" ht="15.5">
-      <c r="A21" s="41"/>
+      <c r="A21" s="56"/>
       <c r="B21" s="13">
         <v>49933</v>
       </c>
@@ -1962,7 +1968,7 @@
       </c>
     </row>
     <row r="22" spans="1:12" ht="15.5">
-      <c r="A22" s="41"/>
+      <c r="A22" s="56"/>
       <c r="B22" s="13">
         <v>49934</v>
       </c>
@@ -1998,7 +2004,7 @@
       </c>
     </row>
     <row r="23" spans="1:12" ht="15.5">
-      <c r="A23" s="41"/>
+      <c r="A23" s="56"/>
       <c r="B23" s="13">
         <v>49935</v>
       </c>
@@ -2034,7 +2040,7 @@
       </c>
     </row>
     <row r="24" spans="1:12" ht="15.5">
-      <c r="A24" s="41"/>
+      <c r="A24" s="56"/>
       <c r="B24" s="13">
         <v>49936</v>
       </c>
@@ -2070,7 +2076,7 @@
       </c>
     </row>
     <row r="25" spans="1:12" ht="15.5">
-      <c r="A25" s="41"/>
+      <c r="A25" s="56"/>
       <c r="B25" s="13">
         <v>49937</v>
       </c>
@@ -2106,7 +2112,7 @@
       </c>
     </row>
     <row r="26" spans="1:12" ht="15.5">
-      <c r="A26" s="41"/>
+      <c r="A26" s="56"/>
       <c r="B26" s="13">
         <v>49938</v>
       </c>
@@ -2142,7 +2148,7 @@
       </c>
     </row>
     <row r="27" spans="1:12" ht="15.5">
-      <c r="A27" s="41"/>
+      <c r="A27" s="56"/>
       <c r="B27" s="13">
         <v>49939</v>
       </c>
@@ -2178,7 +2184,7 @@
       </c>
     </row>
     <row r="28" spans="1:12" ht="15.5">
-      <c r="A28" s="41"/>
+      <c r="A28" s="56"/>
       <c r="B28" s="13">
         <v>49940</v>
       </c>
@@ -2214,7 +2220,7 @@
       </c>
     </row>
     <row r="29" spans="1:12" ht="15.5">
-      <c r="A29" s="41"/>
+      <c r="A29" s="56"/>
       <c r="B29" s="13">
         <v>49941</v>
       </c>
@@ -2250,7 +2256,7 @@
       </c>
     </row>
     <row r="30" spans="1:12" ht="15.5">
-      <c r="A30" s="41"/>
+      <c r="A30" s="56"/>
       <c r="B30" s="13">
         <v>49942</v>
       </c>
@@ -2286,22 +2292,22 @@
       </c>
     </row>
     <row r="31" spans="1:12" ht="31">
-      <c r="A31" s="57"/>
-      <c r="B31" s="58"/>
-      <c r="C31" s="59"/>
-      <c r="D31" s="60"/>
-      <c r="E31" s="61"/>
+      <c r="A31" s="44"/>
+      <c r="B31" s="45"/>
+      <c r="C31" s="46"/>
+      <c r="D31" s="47"/>
+      <c r="E31" s="48"/>
       <c r="F31" s="27"/>
-      <c r="G31" s="62"/>
-      <c r="H31" s="63"/>
-      <c r="I31" s="54" t="s">
+      <c r="G31" s="49"/>
+      <c r="H31" s="50"/>
+      <c r="I31" s="58" t="s">
         <v>23</v>
       </c>
-      <c r="J31" s="64"/>
-      <c r="K31" s="55">
+      <c r="J31" s="51"/>
+      <c r="K31" s="59">
         <v>9727.5</v>
       </c>
-      <c r="L31" s="56">
+      <c r="L31" s="60">
         <v>2279.8249999999998</v>
       </c>
     </row>

</xml_diff>